<commit_message>
Add offline signage size FAQ
</commit_message>
<xml_diff>
--- a/darang/faq/ipark_faq_dataset_admin_v2.xlsx
+++ b/darang/faq/ipark_faq_dataset_admin_v2.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA52"/>
+  <dimension ref="A1:AA53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3664,12 +3664,12 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>8.6</t>
+          <t>8.12</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>매장 운영 및 서비스 기준</t>
+          <t>POS</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -4664,12 +4664,12 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>8.7</t>
+          <t>8.13</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>매장 비품/쇼핑백/내선전화/POS</t>
+          <t>유선전화</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -4789,12 +4789,12 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>8.7</t>
+          <t>8.12</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>매장 비품/쇼핑백/내선전화/POS</t>
+          <t>POS</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -4914,12 +4914,12 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>8.7</t>
+          <t>8.12</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>매장 비품/쇼핑백/내선전화/POS</t>
+          <t>POS</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -7018,6 +7018,153 @@
       <c r="AA52" s="3" t="inlineStr">
         <is>
           <t>답변 입력용 표.xls; 브랜드faq_BRD.md; kakaodata</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>FAQ-052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>8.10</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>???, ???, ??? ??</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>???? ??? ??? ?????.</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>???? ??? ??? ?????.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>???? ??? ?? ???? ?????.</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>???? ???? ??? ??? ??? ????</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>??? ??? ?? ???? ???? ????.</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>??? ??? ???? ?????.</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>??? ???? ??? ??? ??? ???.</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>????, ??, ??? ??? ??? ????</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>???? ???? mm ???? ? ? ?????</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>???? ??? ??? ?????.; ???? ??? ?? ???? ?????.; ???? ???? ??? ??? ??? ????; ??? ??? ?? ???? ???? ????.; ??? ??? ???? ?????.; ??? ???? ??? ??? ??? ???.; ????, ??, ??? ??? ??? ????; ???? ???? mm ???? ? ? ?????; ??? ?? ?? ??? ??? ???? ????.; ???? ??? ??? ??? ?????.</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>???? ???? ?? ???(mm) ???? ????? ???.
+[???]
+CGV ???(2? 1 SET)
+- ???? ??: 833*1,965
+- ?????? ??: 833*1,760
+EV ??: 1,000*500
+ES ??: 1,100*700
+??1F ????: 2,910*3,240
+?????: 365*1,100
+[???]
+3F ???? ? ??
+- ?????: 3,011*2,119
+- ?????: 1,375*2,075
+4F ???? ????: 1,800*400
+4F ???? ? ?? ???: 3,204*3,188
+4F ???? ???
+- ????: 1,800*400
+- ??? ??: 350*1,400
+4F ?? ???(??): 1,200*400
+6F ? ??
+- ????: 1,800*400
+- ?? ???: ? 400*2,970 / ? 410*2,970
+6F ???/???? ????: 1,200*400</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>?? ??? ?? ???? ?? ???? ?, ?? ??? ?? ?? ??? ??? ?? ????? ????? ???.</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>?? ???</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>?? ??? ??? ?? ??? ?? ?? ?? ??? ??? ? ????.</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>?? ??? ??</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>?? ?</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr"/>
+      <c r="X53" t="inlineStr"/>
+      <c r="Y53" t="inlineStr"/>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>?? ?? ???? ??? ??? ??</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove PMS from contact channels
</commit_message>
<xml_diff>
--- a/darang/faq/ipark_faq_dataset_admin_v2.xlsx
+++ b/darang/faq/ipark_faq_dataset_admin_v2.xlsx
@@ -1234,7 +1234,7 @@
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>PMS(https://pms.iparkmall.co.kr/intro); 보안 02-2012-4112</t>
+          <t>보안 02-2012-4112</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t>PMS(https://pms.iparkmall.co.kr/intro); 보안 02-2012-4112</t>
+          <t>보안 02-2012-4112</t>
         </is>
       </c>
       <c r="S7" s="4" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>PMS(https://pms.iparkmall.co.kr/intro); 보안 02-2012-4112</t>
+          <t>보안 02-2012-4112</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>PMS(https://pms.iparkmall.co.kr/intro); 보안 02-2012-4112</t>
+          <t>보안 02-2012-4112</t>
         </is>
       </c>
       <c r="S9" s="4" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
-          <t>PMS(https://pms.iparkmall.co.kr/intro); 보안 02-2012-4112</t>
+          <t>보안 02-2012-4112</t>
         </is>
       </c>
       <c r="S10" s="3" t="inlineStr">
@@ -5984,7 +5984,7 @@
       </c>
       <c r="R44" s="3" t="inlineStr">
         <is>
-          <t>담당 바이어; PMS</t>
+          <t>담당 바이어</t>
         </is>
       </c>
       <c r="S44" s="3" t="inlineStr">
@@ -6109,7 +6109,7 @@
       </c>
       <c r="R45" s="4" t="inlineStr">
         <is>
-          <t>담당 바이어; PMS</t>
+          <t>담당 바이어</t>
         </is>
       </c>
       <c r="S45" s="4" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="R46" s="3" t="inlineStr">
         <is>
-          <t>담당 바이어; PMS</t>
+          <t>담당 바이어</t>
         </is>
       </c>
       <c r="S46" s="3" t="inlineStr">
@@ -6359,7 +6359,7 @@
       </c>
       <c r="R47" s="4" t="inlineStr">
         <is>
-          <t>담당 바이어; PMS</t>
+          <t>담당 바이어</t>
         </is>
       </c>
       <c r="S47" s="4" t="inlineStr">
@@ -6484,7 +6484,7 @@
       </c>
       <c r="R48" s="3" t="inlineStr">
         <is>
-          <t>담당 바이어; PMS</t>
+          <t>담당 바이어</t>
         </is>
       </c>
       <c r="S48" s="3" t="inlineStr">
@@ -7154,9 +7154,6 @@
           <t>?? ?</t>
         </is>
       </c>
-      <c r="W53" t="inlineStr"/>
-      <c r="X53" t="inlineStr"/>
-      <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr">
         <is>
           <t>2026-03-16</t>

</xml_diff>

<commit_message>
Fix backend fallback and parking FAQ sync
</commit_message>
<xml_diff>
--- a/darang/faq/ipark_faq_dataset_admin_v2.xlsx
+++ b/darang/faq/ipark_faq_dataset_admin_v2.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA53"/>
+  <dimension ref="A1:AA54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
-          <t>주차 02-2012-0074; 방재 02-2012-0119</t>
+          <t>?? 02-2012-0074; ?? 02-2012-4112</t>
         </is>
       </c>
       <c r="S11" s="4" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
-          <t>주차 02-2012-0074; 방재 02-2012-0119</t>
+          <t>?? 02-2012-0074; ?? 02-2012-4112</t>
         </is>
       </c>
       <c r="S12" s="3" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="R13" s="4" t="inlineStr">
         <is>
-          <t>주차 02-2012-0074; 방재 02-2012-0119</t>
+          <t>?? 02-2012-0074; ?? 02-2012-4112</t>
         </is>
       </c>
       <c r="S13" s="4" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
-          <t>주차 02-2012-0074; 방재 02-2012-0119</t>
+          <t>?? 02-2012-0074; ?? 02-2012-4112</t>
         </is>
       </c>
       <c r="S14" s="3" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>주차 02-2012-0074; 방재 02-2012-0119</t>
+          <t>?? 02-2012-0074; ?? 02-2012-4112</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t>주차 02-2012-0074; 방재 02-2012-0119</t>
+          <t>?? 02-2012-0074; ?? 02-2012-4112</t>
         </is>
       </c>
       <c r="S16" s="3" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>주차 02-2012-0074; 방재 02-2012-0119</t>
+          <t>?? 02-2012-0074; ?? 02-2012-4112</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
@@ -7162,6 +7162,118 @@
       <c r="AA53" t="inlineStr">
         <is>
           <t>?? ?? ???? ??? ??? ??</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>FAQ-053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>????</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>8.3</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>??, ??, ??, ??</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>??? ??? ??????</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>???? ??? ????</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>??? ??? ?????.</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>??? ???? ??? ??? ??????</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>???? ???? ??? ????</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>??? ?? ??????.</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>???? ?? ? ?? ????</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>???? ?? ??? ?? ????</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>??? ?? ??? ??? ???.</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>??? ??? ??????; ???? ??? ????; ??? ??? ?????.; ??? ???? ??? ??? ??????; ???? ???? ??? ????; ??? ?? ??????.; ???? ?? ? ?? ????; ???? ?? ??? ?? ????; ??? ?? ??? ??? ???.; ??? ?? ?? ??????.</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>???? ????? ?? 1? ????? ??? ????. ??? ??? ?? ??? ???? ?? ?? ? ?? 02-2012-4112? ?? ????? ?? ??? ????? ? ????.</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>????? ?? ??? ??? ?????, ??? ?? ?? 02-2012-4112? ??? ?? ??? ?? ????? ???.</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>?? 02-2012-0074; ?? 02-2012-4112</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>?? ??? ??</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>??? ?? ?? FAQ ??</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>?? ??? ?.xls; ???faq_BRD.md; kakaodata</t>
         </is>
       </c>
     </row>

</xml_diff>